<commit_message>
chore: update ERP valuation data and charts
</commit_message>
<xml_diff>
--- a/erp_valuation/erp_portfolio.xlsx
+++ b/erp_valuation/erp_portfolio.xlsx
@@ -3850,43 +3850,43 @@
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>30.83829715602115</v>
+        <v>30.55094326469016</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>11.90371291182457</v>
+        <v>12.18209721752674</v>
       </c>
       <c r="D94" s="2" t="n">
-        <v>25.9799079787846</v>
+        <v>26.2880094123509</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>27.42093054006139</v>
+        <v>27.80232970506856</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>3.734695430199554</v>
+        <v>4.014262795012042</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>7.268286694463483</v>
+        <v>6.663889794340077</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>61.97589888671864</v>
+        <v>63.17624150343</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>25.59983050065752</v>
+        <v>25.46303751324943</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>52.69286460826729</v>
+        <v>52.89301743264895</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>46.41956067373302</v>
+        <v>46.67348631596258</v>
       </c>
       <c r="L94" s="2" t="n">
-        <v>24.745264159472</v>
+        <v>24.78488357549217</v>
       </c>
       <c r="M94" s="2" t="n">
         <v>15</v>
       </c>
       <c r="N94" s="3" t="n">
-        <v>9.745264159472004</v>
+        <v>9.784883575492174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>